<commit_message>
fix(formularios): importador sem falso-verde, com releitura estrita e validacao de itens
Motor, pagamento canonico e GET sem resposta passam a ser pendencia; item sem
nome, nome repetido, janela pos-chaves, permuta zerada, cronograma invalido e
base financiavel ambigua sao barrados antes de escrever. URL exige https e
nao segue redirect; o script de pagamento so aceita estudo qa- ou --forcar.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YboM7dK3kzvHvStTxNRE27
</commit_message>
<xml_diff>
--- a/referencia/formularios/exemplos/exemplo-incorporacao-aurora-parque-avancado.xlsx
+++ b/referencia/formularios/exemplos/exemplo-incorporacao-aurora-parque-avancado.xlsx
@@ -716,7 +716,7 @@
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>lista: manual (inserir novo) | nucleo (buscar terreno)</t>
+          <t>lista: manual (inserir novo) | nucleo (buscar terreno — o importador só aceita manual)</t>
         </is>
       </c>
       <c r="D8" s="8" t="inlineStr">
@@ -6216,7 +6216,7 @@
     <row r="324" ht="117" customHeight="1">
       <c r="A324" s="13" t="inlineStr">
         <is>
-          <t>Categorias e unidades aceitas (rs = R$ · rs_m2_priv = R$/m² privativo · rs_m2_terreno · pct_vgv · pct_receita · pct_obra · pct_recebido · pct_constr). TERRENO: Preço (rs, rs_m2_terreno; permuta financeira: rs, pct_vgv) · Registro (rs, rs_m2_priv) · Outro (rs, pct_vgv). OBRA: Construção, Decoração (rs, rs_m2_priv) · Outorga, Contingência, Outro (rs, pct_vgv) · Gestão da obra (rs, pct_obra). DIRETOS: Marketing &amp; Publicidade, Manutenção pós-obra, Outro (rs, pct_vgv, pct_recebido) · Corretagem de vendas (pct_vgv) · Projetos (rs, rs_m2_priv, pct_constr) · Licenças e Aprovações (rs, rs_m2_priv). INDIRETO: Marketing global, Gestão, Outro (rs, pct_vgv, pct_recebido) · Stand de vendas (rs, pct_vgv). FINANCEIRO: Juros de financiamento, Taxas bancárias, Estruturação de dívida, Investidores, Outro (rs, pct_vgv). Cronograma padrão: terreno/Preço = customizado; terreno/demais, indireto = planejamento; obra/diretos/financeiro = obra; Manutenção pós-obra = pos_obra. Início e Duração só valem com cronograma = customizado; cronograma ancorado em fase customizada = escrever "fase: &lt;nome da fase&gt;". Corretagem sai no mês da venda e a permuta física na entrega das unidades (não escolhem distribuição). Obrigatórias: terreno/Preço, obra/Construção, diretos/Corretagem de vendas (% VGV).</t>
+          <t>Categorias e unidades aceitas (rs = R$ · rs_m2_priv = R$/m² privativo · rs_m2_terreno · pct_vgv · pct_obra · pct_recebido · pct_constr). TERRENO: Preço (rs, rs_m2_terreno; permuta financeira: rs, pct_vgv) · Registro (rs, rs_m2_priv) · Outro (rs, pct_vgv). OBRA: Construção, Decoração (rs, rs_m2_priv) · Outorga, Contingência, Outro (rs, pct_vgv) · Gestão da obra (rs, pct_obra). DIRETOS: Marketing &amp; Publicidade, Manutenção pós-obra, Outro (rs, pct_vgv, pct_recebido) · Corretagem de vendas (pct_vgv) · Projetos (rs, rs_m2_priv, pct_constr) · Licenças e Aprovações (rs, rs_m2_priv). INDIRETO: Marketing global, Gestão, Outro (rs, pct_vgv, pct_recebido) · Stand de vendas (rs, pct_vgv). FINANCEIRO: Juros de financiamento, Taxas bancárias, Estruturação de dívida, Investidores, Outro (rs, pct_vgv). Cronograma padrão: terreno/Preço = customizado; terreno/demais, indireto = planejamento; obra/diretos/financeiro = obra; Manutenção pós-obra = pos_obra. Início e Duração só valem com cronograma = customizado; cronograma ancorado em fase customizada = escrever "fase: &lt;nome da fase&gt;". Corretagem sai no mês da venda e a permuta física na entrega das unidades (não escolhem distribuição). Obrigatórias: terreno/Preço, obra/Construção, diretos/Corretagem de vendas (% VGV).</t>
         </is>
       </c>
     </row>
@@ -6313,7 +6313,7 @@
       </c>
       <c r="C330" s="7" t="inlineStr">
         <is>
-          <t>lista: rs | rs_m2_priv | rs_m2_terreno | pct_vgv | pct_receita | pct_obra | pct_recebido | pct_constr</t>
+          <t>lista: rs | rs_m2_priv | rs_m2_terreno | pct_vgv | pct_obra | pct_recebido | pct_constr</t>
         </is>
       </c>
       <c r="D330" s="8" t="inlineStr">
@@ -6524,7 +6524,7 @@
       </c>
       <c r="C341" s="7" t="inlineStr">
         <is>
-          <t>lista: rs | rs_m2_priv | rs_m2_terreno | pct_vgv | pct_receita | pct_obra | pct_recebido | pct_constr</t>
+          <t>lista: rs | rs_m2_priv | rs_m2_terreno | pct_vgv | pct_obra | pct_recebido | pct_constr</t>
         </is>
       </c>
       <c r="D341" s="8" t="inlineStr">
@@ -6731,7 +6731,7 @@
       </c>
       <c r="C352" s="7" t="inlineStr">
         <is>
-          <t>lista: rs | rs_m2_priv | rs_m2_terreno | pct_vgv | pct_receita | pct_obra | pct_recebido | pct_constr</t>
+          <t>lista: rs | rs_m2_priv | rs_m2_terreno | pct_vgv | pct_obra | pct_recebido | pct_constr</t>
         </is>
       </c>
       <c r="D352" s="8" t="inlineStr">
@@ -6930,7 +6930,7 @@
       </c>
       <c r="C363" s="7" t="inlineStr">
         <is>
-          <t>lista: rs | rs_m2_priv | rs_m2_terreno | pct_vgv | pct_receita | pct_obra | pct_recebido | pct_constr</t>
+          <t>lista: rs | rs_m2_priv | rs_m2_terreno | pct_vgv | pct_obra | pct_recebido | pct_constr</t>
         </is>
       </c>
       <c r="D363" s="8" t="inlineStr">
@@ -7141,7 +7141,7 @@
       </c>
       <c r="C374" s="7" t="inlineStr">
         <is>
-          <t>lista: rs | rs_m2_priv | rs_m2_terreno | pct_vgv | pct_receita | pct_obra | pct_recebido | pct_constr</t>
+          <t>lista: rs | rs_m2_priv | rs_m2_terreno | pct_vgv | pct_obra | pct_recebido | pct_constr</t>
         </is>
       </c>
       <c r="D374" s="8" t="inlineStr">
@@ -7352,7 +7352,7 @@
       </c>
       <c r="C385" s="7" t="inlineStr">
         <is>
-          <t>lista: rs | rs_m2_priv | rs_m2_terreno | pct_vgv | pct_receita | pct_obra | pct_recebido | pct_constr</t>
+          <t>lista: rs | rs_m2_priv | rs_m2_terreno | pct_vgv | pct_obra | pct_recebido | pct_constr</t>
         </is>
       </c>
       <c r="D385" s="8" t="inlineStr">
@@ -7563,7 +7563,7 @@
       </c>
       <c r="C396" s="7" t="inlineStr">
         <is>
-          <t>lista: rs | rs_m2_priv | rs_m2_terreno | pct_vgv | pct_receita | pct_obra | pct_recebido | pct_constr</t>
+          <t>lista: rs | rs_m2_priv | rs_m2_terreno | pct_vgv | pct_obra | pct_recebido | pct_constr</t>
         </is>
       </c>
       <c r="D396" s="8" t="inlineStr">
@@ -7770,7 +7770,7 @@
       </c>
       <c r="C407" s="7" t="inlineStr">
         <is>
-          <t>lista: rs | rs_m2_priv | rs_m2_terreno | pct_vgv | pct_receita | pct_obra | pct_recebido | pct_constr</t>
+          <t>lista: rs | rs_m2_priv | rs_m2_terreno | pct_vgv | pct_obra | pct_recebido | pct_constr</t>
         </is>
       </c>
       <c r="D407" s="8" t="inlineStr">
@@ -7977,7 +7977,7 @@
       </c>
       <c r="C418" s="7" t="inlineStr">
         <is>
-          <t>lista: rs | rs_m2_priv | rs_m2_terreno | pct_vgv | pct_receita | pct_obra | pct_recebido | pct_constr</t>
+          <t>lista: rs | rs_m2_priv | rs_m2_terreno | pct_vgv | pct_obra | pct_recebido | pct_constr</t>
         </is>
       </c>
       <c r="D418" s="8" t="inlineStr">
@@ -8184,7 +8184,7 @@
       </c>
       <c r="C429" s="7" t="inlineStr">
         <is>
-          <t>lista: rs | rs_m2_priv | rs_m2_terreno | pct_vgv | pct_receita | pct_obra | pct_recebido | pct_constr</t>
+          <t>lista: rs | rs_m2_priv | rs_m2_terreno | pct_vgv | pct_obra | pct_recebido | pct_constr</t>
         </is>
       </c>
       <c r="D429" s="8" t="inlineStr">
@@ -8391,7 +8391,7 @@
       </c>
       <c r="C440" s="7" t="inlineStr">
         <is>
-          <t>lista: rs | rs_m2_priv | rs_m2_terreno | pct_vgv | pct_receita | pct_obra | pct_recebido | pct_constr</t>
+          <t>lista: rs | rs_m2_priv | rs_m2_terreno | pct_vgv | pct_obra | pct_recebido | pct_constr</t>
         </is>
       </c>
       <c r="D440" s="8" t="inlineStr">
@@ -8590,7 +8590,7 @@
       <c r="B451" s="6" t="n"/>
       <c r="C451" s="7" t="inlineStr">
         <is>
-          <t>lista: rs | rs_m2_priv | rs_m2_terreno | pct_vgv | pct_receita | pct_obra | pct_recebido | pct_constr</t>
+          <t>lista: rs | rs_m2_priv | rs_m2_terreno | pct_vgv | pct_obra | pct_recebido | pct_constr</t>
         </is>
       </c>
       <c r="D451" s="8" t="inlineStr">
@@ -8775,7 +8775,7 @@
       <c r="B462" s="6" t="n"/>
       <c r="C462" s="7" t="inlineStr">
         <is>
-          <t>lista: rs | rs_m2_priv | rs_m2_terreno | pct_vgv | pct_receita | pct_obra | pct_recebido | pct_constr</t>
+          <t>lista: rs | rs_m2_priv | rs_m2_terreno | pct_vgv | pct_obra | pct_recebido | pct_constr</t>
         </is>
       </c>
       <c r="D462" s="8" t="inlineStr">
@@ -8960,7 +8960,7 @@
       <c r="B473" s="6" t="n"/>
       <c r="C473" s="7" t="inlineStr">
         <is>
-          <t>lista: rs | rs_m2_priv | rs_m2_terreno | pct_vgv | pct_receita | pct_obra | pct_recebido | pct_constr</t>
+          <t>lista: rs | rs_m2_priv | rs_m2_terreno | pct_vgv | pct_obra | pct_recebido | pct_constr</t>
         </is>
       </c>
       <c r="D473" s="8" t="inlineStr">
@@ -9145,7 +9145,7 @@
       <c r="B484" s="6" t="n"/>
       <c r="C484" s="7" t="inlineStr">
         <is>
-          <t>lista: rs | rs_m2_priv | rs_m2_terreno | pct_vgv | pct_receita | pct_obra | pct_recebido | pct_constr</t>
+          <t>lista: rs | rs_m2_priv | rs_m2_terreno | pct_vgv | pct_obra | pct_recebido | pct_constr</t>
         </is>
       </c>
       <c r="D484" s="8" t="inlineStr">
@@ -9330,7 +9330,7 @@
       <c r="B495" s="6" t="n"/>
       <c r="C495" s="7" t="inlineStr">
         <is>
-          <t>lista: rs | rs_m2_priv | rs_m2_terreno | pct_vgv | pct_receita | pct_obra | pct_recebido | pct_constr</t>
+          <t>lista: rs | rs_m2_priv | rs_m2_terreno | pct_vgv | pct_obra | pct_recebido | pct_constr</t>
         </is>
       </c>
       <c r="D495" s="8" t="inlineStr">
@@ -9515,7 +9515,7 @@
       <c r="B506" s="6" t="n"/>
       <c r="C506" s="7" t="inlineStr">
         <is>
-          <t>lista: rs | rs_m2_priv | rs_m2_terreno | pct_vgv | pct_receita | pct_obra | pct_recebido | pct_constr</t>
+          <t>lista: rs | rs_m2_priv | rs_m2_terreno | pct_vgv | pct_obra | pct_recebido | pct_constr</t>
         </is>
       </c>
       <c r="D506" s="8" t="inlineStr">
@@ -9700,7 +9700,7 @@
       <c r="B517" s="6" t="n"/>
       <c r="C517" s="7" t="inlineStr">
         <is>
-          <t>lista: rs | rs_m2_priv | rs_m2_terreno | pct_vgv | pct_receita | pct_obra | pct_recebido | pct_constr</t>
+          <t>lista: rs | rs_m2_priv | rs_m2_terreno | pct_vgv | pct_obra | pct_recebido | pct_constr</t>
         </is>
       </c>
       <c r="D517" s="8" t="inlineStr">
@@ -9885,7 +9885,7 @@
       <c r="B528" s="6" t="n"/>
       <c r="C528" s="7" t="inlineStr">
         <is>
-          <t>lista: rs | rs_m2_priv | rs_m2_terreno | pct_vgv | pct_receita | pct_obra | pct_recebido | pct_constr</t>
+          <t>lista: rs | rs_m2_priv | rs_m2_terreno | pct_vgv | pct_obra | pct_recebido | pct_constr</t>
         </is>
       </c>
       <c r="D528" s="8" t="inlineStr">
@@ -10070,7 +10070,7 @@
       <c r="B539" s="6" t="n"/>
       <c r="C539" s="7" t="inlineStr">
         <is>
-          <t>lista: rs | rs_m2_priv | rs_m2_terreno | pct_vgv | pct_receita | pct_obra | pct_recebido | pct_constr</t>
+          <t>lista: rs | rs_m2_priv | rs_m2_terreno | pct_vgv | pct_obra | pct_recebido | pct_constr</t>
         </is>
       </c>
       <c r="D539" s="8" t="inlineStr">
@@ -10255,7 +10255,7 @@
       <c r="B550" s="6" t="n"/>
       <c r="C550" s="7" t="inlineStr">
         <is>
-          <t>lista: rs | rs_m2_priv | rs_m2_terreno | pct_vgv | pct_receita | pct_obra | pct_recebido | pct_constr</t>
+          <t>lista: rs | rs_m2_priv | rs_m2_terreno | pct_vgv | pct_obra | pct_recebido | pct_constr</t>
         </is>
       </c>
       <c r="D550" s="8" t="inlineStr">
@@ -10440,7 +10440,7 @@
       <c r="B561" s="6" t="n"/>
       <c r="C561" s="7" t="inlineStr">
         <is>
-          <t>lista: rs | rs_m2_priv | rs_m2_terreno | pct_vgv | pct_receita | pct_obra | pct_recebido | pct_constr</t>
+          <t>lista: rs | rs_m2_priv | rs_m2_terreno | pct_vgv | pct_obra | pct_recebido | pct_constr</t>
         </is>
       </c>
       <c r="D561" s="8" t="inlineStr">
@@ -10625,7 +10625,7 @@
       <c r="B572" s="6" t="n"/>
       <c r="C572" s="7" t="inlineStr">
         <is>
-          <t>lista: rs | rs_m2_priv | rs_m2_terreno | pct_vgv | pct_receita | pct_obra | pct_recebido | pct_constr</t>
+          <t>lista: rs | rs_m2_priv | rs_m2_terreno | pct_vgv | pct_obra | pct_recebido | pct_constr</t>
         </is>
       </c>
       <c r="D572" s="8" t="inlineStr">
@@ -10810,7 +10810,7 @@
       <c r="B583" s="6" t="n"/>
       <c r="C583" s="7" t="inlineStr">
         <is>
-          <t>lista: rs | rs_m2_priv | rs_m2_terreno | pct_vgv | pct_receita | pct_obra | pct_recebido | pct_constr</t>
+          <t>lista: rs | rs_m2_priv | rs_m2_terreno | pct_vgv | pct_obra | pct_recebido | pct_constr</t>
         </is>
       </c>
       <c r="D583" s="8" t="inlineStr">
@@ -10995,7 +10995,7 @@
       <c r="B594" s="6" t="n"/>
       <c r="C594" s="7" t="inlineStr">
         <is>
-          <t>lista: rs | rs_m2_priv | rs_m2_terreno | pct_vgv | pct_receita | pct_obra | pct_recebido | pct_constr</t>
+          <t>lista: rs | rs_m2_priv | rs_m2_terreno | pct_vgv | pct_obra | pct_recebido | pct_constr</t>
         </is>
       </c>
       <c r="D594" s="8" t="inlineStr">
@@ -11180,7 +11180,7 @@
       <c r="B605" s="6" t="n"/>
       <c r="C605" s="7" t="inlineStr">
         <is>
-          <t>lista: rs | rs_m2_priv | rs_m2_terreno | pct_vgv | pct_receita | pct_obra | pct_recebido | pct_constr</t>
+          <t>lista: rs | rs_m2_priv | rs_m2_terreno | pct_vgv | pct_obra | pct_recebido | pct_constr</t>
         </is>
       </c>
       <c r="D605" s="8" t="inlineStr">
@@ -11365,7 +11365,7 @@
       <c r="B616" s="6" t="n"/>
       <c r="C616" s="7" t="inlineStr">
         <is>
-          <t>lista: rs | rs_m2_priv | rs_m2_terreno | pct_vgv | pct_receita | pct_obra | pct_recebido | pct_constr</t>
+          <t>lista: rs | rs_m2_priv | rs_m2_terreno | pct_vgv | pct_obra | pct_recebido | pct_constr</t>
         </is>
       </c>
       <c r="D616" s="8" t="inlineStr">
@@ -11550,7 +11550,7 @@
       <c r="B627" s="6" t="n"/>
       <c r="C627" s="7" t="inlineStr">
         <is>
-          <t>lista: rs | rs_m2_priv | rs_m2_terreno | pct_vgv | pct_receita | pct_obra | pct_recebido | pct_constr</t>
+          <t>lista: rs | rs_m2_priv | rs_m2_terreno | pct_vgv | pct_obra | pct_recebido | pct_constr</t>
         </is>
       </c>
       <c r="D627" s="8" t="inlineStr">
@@ -17513,7 +17513,7 @@
       <formula1>"Entrada,Parcelamento"</formula1>
     </dataValidation>
     <dataValidation sqref="B330 B341 B363 B374 B385 B396 B407 B418 B429 B440 B451 B462 B473 B484 B495 B506 B517 B528 B539 B550 B561 B572 B583 B594 B605 B616 B627" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor inválido" error="Escolha um valor da lista." type="list">
-      <formula1>"rs,rs_m2_priv,rs_m2_terreno,pct_vgv,pct_receita,pct_obra,pct_recebido,pct_constr"</formula1>
+      <formula1>"rs,rs_m2_priv,rs_m2_terreno,pct_vgv,pct_obra,pct_recebido,pct_constr"</formula1>
     </dataValidation>
     <dataValidation sqref="B332 B343 B354 B365 B376 B387 B398 B409 B420 B431 B442 B453 B464 B475 B486 B497 B508 B519 B530 B541 B552 B563 B574 B585 B596 B607 B618 B629" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Confira o valor" error="Valor fora da faixa esperada (0 a 10)." type="decimal" errorStyle="warning" operator="between">
       <formula1>0</formula1>

</xml_diff>

<commit_message>
fix(formularios): observações da rodada 1 da revisão
- nota da seção 6 cita a venda feita depois da entrega;
- validação de dados da carteira cedida passa a recusar 0%, como o importador;
- releitura ignora participação de até meio centésimo dos dois lados;
- PROGRESSO diz que 40/60 é do saldo de chaves.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0144wHVsWbipSxm6TLMMago3
</commit_message>
<xml_diff>
--- a/referencia/formularios/exemplos/exemplo-incorporacao-aurora-parque-avancado.xlsx
+++ b/referencia/formularios/exemplos/exemplo-incorporacao-aurora-parque-avancado.xlsx
@@ -3225,7 +3225,7 @@
     <row r="150" ht="39" customHeight="1">
       <c r="A150" s="13" t="inlineStr">
         <is>
-          <t>Saldo de chaves = o Repasse acima. "Repasse bancário" é a parte dele paga pelo banco no mês seguinte ao fim da obra (vazio = 100%, tudo no banco). O resto vira carteira própria: a empresa financia o comprador em N parcelas mensais Price com os Juros de tabela, a partir do mês seguinte ao fim da obra + a carência. Loteamento sem banco: 0%.</t>
+          <t>Saldo de chaves = o Repasse acima. "Repasse bancário" é a parte dele paga pelo banco no mês seguinte ao fim da obra (vazio = 100%, tudo no banco). O resto vira carteira própria: a empresa financia o comprador em N parcelas mensais Price com os Juros de tabela, a partir do mês seguinte ao fim da obra + a carência (nunca antes do mês seguinte à venda): também a venda feita depois da entrega tem essa parte financiada. Loteamento sem banco: 0%.</t>
         </is>
       </c>
     </row>
@@ -18313,7 +18313,7 @@
     <mergeCell ref="A562:D562"/>
     <mergeCell ref="A151:D151"/>
   </mergeCells>
-  <dataValidations count="24">
+  <dataValidations count="25">
     <dataValidation sqref="B5 B14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="No máximo 200 caracteres." type="textLength" errorStyle="warning" operator="lessThanOrEqual">
       <formula1>200</formula1>
     </dataValidation>
@@ -18334,7 +18334,7 @@
       <formula1>0</formula1>
       <formula2>9.9999</formula2>
     </dataValidation>
-    <dataValidation sqref="B22 B25 B153 B154 B155 B159 B164 B165 B166 B170 B175 B176 B177 B181 B186 B187 B188 B192 B197 B198 B199 B203 B211 B213 B214 B219 B221 B222 B227 B229 B230 B235 B237 B238 B243 B245 B246 B251 B253 B254 B259 B261 B262 B267 B269 B270 B275 B277 B278 B283 B285 B286 B658 B663 B671 B672 B673 B683 B686 B696 B699 B709 B712 B721 B728 B735 B741 B742 B743 B750 B751 B752 B759 B760 B761" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Confira o valor" error="Valor fora da faixa esperada (0 a 1)." type="decimal" errorStyle="warning" operator="between">
+    <dataValidation sqref="B22 B25 B153 B154 B155 B159 B164 B165 B166 B170 B175 B176 B177 B181 B186 B187 B188 B192 B197 B198 B199 B203 B211 B213 B214 B219 B221 B222 B227 B229 B230 B235 B237 B238 B243 B245 B246 B251 B253 B254 B259 B261 B262 B267 B269 B270 B275 B277 B278 B283 B285 B286 B658 B663 B671 B672 B673 B683 B686 B696 B699 B709 B712 B721 B728 B735 B742 B743 B751 B752 B760 B761" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Confira o valor" error="Valor fora da faixa esperada (0 a 1)." type="decimal" errorStyle="warning" operator="between">
       <formula1>0</formula1>
       <formula2>1</formula2>
     </dataValidation>
@@ -18390,6 +18390,10 @@
     <dataValidation sqref="B720 B727 B734" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor inválido" error="Escolha um valor da lista." type="list">
       <formula1>"permuta_financeira,resultado_final"</formula1>
     </dataValidation>
+    <dataValidation sqref="B741 B750 B759" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Confira o valor" error="Valor fora da faixa esperada (0.0001 a 1)." type="decimal" errorStyle="warning" operator="between">
+      <formula1>0.0001</formula1>
+      <formula2>1</formula2>
+    </dataValidation>
     <dataValidation sqref="B766 B767 B769 B770 B772 B773 B775 B776 B778 B779" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Confira o valor" error="Valor fora da faixa esperada (-1 a 10)." type="decimal" errorStyle="warning" operator="between">
       <formula1>-1</formula1>
       <formula2>10</formula2>

</xml_diff>